<commit_message>
Traer datos de PBI desde el año 2000
Cambia el rango de la API del Banco Mundial de los ultimos 5 anios a
date=2000:2025, y regenera el CSV/XLSX con la serie completa.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/pbi_argentina.xlsx
+++ b/pbi_argentina.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -436,63 +436,336 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2021</t>
+          <t>2000</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>486564085480.036</v>
+        <v>284203750000</v>
       </c>
       <c r="C2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2022</t>
+          <t>2001</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>633993756301.08</v>
+        <v>268696750000</v>
       </c>
       <c r="C3" t="n">
-        <v>30.30015474232799</v>
+        <v>-5.456296758927359</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2002</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>649461687959.174</v>
+        <v>97724004251.8602</v>
       </c>
       <c r="C4" t="n">
-        <v>2.439760881611641</v>
+        <v>-63.6303735523931</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2003</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>638365455340.04</v>
+        <v>127586973492.177</v>
       </c>
       <c r="C5" t="n">
-        <v>-1.708527666043236</v>
+        <v>30.55847892126089</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t>2004</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>164657930452.787</v>
+      </c>
+      <c r="C6" t="n">
+        <v>29.05544033684833</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2005</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>198737095012.282</v>
+      </c>
+      <c r="C7" t="n">
+        <v>20.69694697715558</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2006</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>232557260817.308</v>
+      </c>
+      <c r="C8" t="n">
+        <v>17.01754058694272</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2007</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>287530508430.568</v>
+      </c>
+      <c r="C9" t="n">
+        <v>23.63858579175724</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2008</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>361558037110.419</v>
+      </c>
+      <c r="C10" t="n">
+        <v>25.74597356082893</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2009</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>332976484577.619</v>
+      </c>
+      <c r="C11" t="n">
+        <v>-7.905107783310383</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2010</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>423627422092.49</v>
+      </c>
+      <c r="C12" t="n">
+        <v>27.22442626237158</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2011</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>530158122010.442</v>
+      </c>
+      <c r="C13" t="n">
+        <v>25.14726251472297</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2012</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>545982375701.128</v>
+      </c>
+      <c r="C14" t="n">
+        <v>2.984817742804347</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2013</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>552025140252.246</v>
+      </c>
+      <c r="C15" t="n">
+        <v>1.106769159601195</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2014</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>526319673731.638</v>
+      </c>
+      <c r="C16" t="n">
+        <v>-4.656575334388203</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2015</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>594749285413.212</v>
+      </c>
+      <c r="C17" t="n">
+        <v>13.0015302670341</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2016</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>557532320662.955</v>
+      </c>
+      <c r="C18" t="n">
+        <v>-6.257588813141657</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2017</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>643628393281.364</v>
+      </c>
+      <c r="C19" t="n">
+        <v>15.44234646630589</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2018</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>524819892360.176</v>
+      </c>
+      <c r="C20" t="n">
+        <v>-18.45917646912299</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>447754683615.225</v>
+      </c>
+      <c r="C21" t="n">
+        <v>-14.68412494777587</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>385740508436.965</v>
+      </c>
+      <c r="C22" t="n">
+        <v>-13.85003383494507</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>486564085480.036</v>
+      </c>
+      <c r="C23" t="n">
+        <v>26.13766893490441</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>633993756301.08</v>
+      </c>
+      <c r="C24" t="n">
+        <v>30.30015474232799</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>649461687959.174</v>
+      </c>
+      <c r="C25" t="n">
+        <v>2.439760881611641</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>638365455340.04</v>
+      </c>
+      <c r="C26" t="n">
+        <v>-1.708527666043236</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="B6" t="n">
+      <c r="B27" t="n">
         <v>683097891618.597</v>
       </c>
-      <c r="C6" t="n">
+      <c r="C27" t="n">
         <v>7.007339746278918</v>
       </c>
     </row>

</xml_diff>